<commit_message>
Support 5 vœux « sans », priorité sur « avec », capacité dure et sortie .xlsm
- Algorithme : champs sans1..sans5 (au lieu de sans1/sans2), tous pondérés à
  1000 et prioritaires sur les « avec » (500). Constantes AVEC_FIELDS/SANS_FIELDS.
- capacité : plafond DUR robuste — corrige le crash « Impossible de répartir »
  quand toutes les classes ont une capacité saisie ; erreur claire si places
  insuffisantes.
- Sortie : génère assignments_desanonymiser.xlsm avec le projet VBA
  « Desanonymiser » incrusté + onglet diccionari vide (nom_real/id_anonim).
- .bas Anonymiser/Desanonymiser : ajout des en-têtes sans3/sans4/sans5.
- Tests : 5 vœux sans, priorité sans>avec, capacité dure (3 cas). 15/15 OK.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Liste.xlsx
+++ b/Liste.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jordiordonezadellach/Desktop/Projectes/Classes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2388E678-873D-E748-AA77-C5A051FA4437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA63A642-63F1-2D42-98A0-F1582E336B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1840" yWindow="-20560" windowWidth="28040" windowHeight="15820" xr2:uid="{B5B86117-F7DA-9D45-88D5-7A78429F12FC}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="classes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">liste!$A$1:$N$234</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">liste!$A$1:$O$234</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="263">
   <si>
     <t>Elèves à affecter</t>
   </si>
@@ -819,14 +819,20 @@
     <t>Origine</t>
   </si>
   <si>
-    <t>1+H140</t>
+    <t>sans3</t>
+  </si>
+  <si>
+    <t>sans4</t>
+  </si>
+  <si>
+    <t>sans5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -957,6 +963,12 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1680,10 +1692,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{041A12D7-D1F2-5E4A-959D-815F4F1F9005}">
-  <dimension ref="A1:O234"/>
+  <dimension ref="A1:R234"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1727,10 +1739,19 @@
         <v>10</v>
       </c>
       <c r="O1" t="s">
+        <v>260</v>
+      </c>
+      <c r="P1" t="s">
+        <v>261</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>262</v>
+      </c>
+      <c r="R1" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1770,11 +1791,20 @@
       <c r="M2" t="s">
         <v>15</v>
       </c>
-      <c r="O2" t="s">
+      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>15</v>
+      </c>
+      <c r="R2" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1805,14 +1835,14 @@
       <c r="J3">
         <v>2</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>13</v>
       </c>
-      <c r="O3" t="s">
+      <c r="R3" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1843,11 +1873,11 @@
       <c r="J4">
         <v>3</v>
       </c>
-      <c r="O4" t="s">
+      <c r="R4" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1878,11 +1908,11 @@
       <c r="J5">
         <v>1</v>
       </c>
-      <c r="O5" t="s">
+      <c r="R5" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1922,11 +1952,20 @@
       <c r="M6" t="s">
         <v>23</v>
       </c>
-      <c r="O6" t="s">
+      <c r="N6" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R6" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1957,14 +1996,14 @@
       <c r="J7">
         <v>2</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>21</v>
       </c>
-      <c r="O7" t="s">
+      <c r="R7" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1995,11 +2034,11 @@
       <c r="J8">
         <v>2</v>
       </c>
-      <c r="O8" t="s">
+      <c r="R8" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -2030,11 +2069,11 @@
       <c r="J9">
         <v>1</v>
       </c>
-      <c r="O9" t="s">
+      <c r="R9" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -2065,11 +2104,11 @@
       <c r="J10">
         <v>2</v>
       </c>
-      <c r="O10" t="s">
+      <c r="R10" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -2109,11 +2148,20 @@
       <c r="M11" t="s">
         <v>29</v>
       </c>
-      <c r="O11" t="s">
+      <c r="N11" t="s">
+        <v>29</v>
+      </c>
+      <c r="P11" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>29</v>
+      </c>
+      <c r="R11" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -2130,7 +2178,7 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -2144,11 +2192,11 @@
       <c r="J12">
         <v>2</v>
       </c>
-      <c r="O12" t="s">
+      <c r="R12" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -2179,11 +2227,11 @@
       <c r="J13">
         <v>2</v>
       </c>
-      <c r="O13" t="s">
+      <c r="R13" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -2223,11 +2271,20 @@
       <c r="M14" t="s">
         <v>33</v>
       </c>
-      <c r="O14" t="s">
+      <c r="N14" t="s">
+        <v>33</v>
+      </c>
+      <c r="P14" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>33</v>
+      </c>
+      <c r="R14" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -2267,11 +2324,20 @@
       <c r="M15" t="s">
         <v>37</v>
       </c>
-      <c r="O15" t="s">
+      <c r="N15" t="s">
+        <v>37</v>
+      </c>
+      <c r="P15" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>37</v>
+      </c>
+      <c r="R15" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -2302,11 +2368,11 @@
       <c r="J16">
         <v>2</v>
       </c>
-      <c r="O16" t="s">
+      <c r="R16" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -2337,14 +2403,14 @@
       <c r="J17">
         <v>1</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>33</v>
       </c>
-      <c r="O17" t="s">
+      <c r="R17" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2375,11 +2441,11 @@
       <c r="J18">
         <v>1</v>
       </c>
-      <c r="O18" t="s">
+      <c r="R18" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -2410,11 +2476,11 @@
       <c r="J19">
         <v>1</v>
       </c>
-      <c r="O19" t="s">
+      <c r="R19" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -2445,11 +2511,11 @@
       <c r="J20">
         <v>1</v>
       </c>
-      <c r="O20" t="s">
+      <c r="R20" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -2490,13 +2556,22 @@
         <v>42</v>
       </c>
       <c r="N21" t="s">
+        <v>42</v>
+      </c>
+      <c r="O21" t="s">
         <v>43</v>
       </c>
-      <c r="O21" t="s">
+      <c r="P21" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>42</v>
+      </c>
+      <c r="R21" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -2527,11 +2602,11 @@
       <c r="J22">
         <v>1</v>
       </c>
-      <c r="O22" t="s">
+      <c r="R22" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -2562,11 +2637,11 @@
       <c r="J23">
         <v>2</v>
       </c>
-      <c r="O23" t="s">
+      <c r="R23" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -2597,14 +2672,14 @@
       <c r="J24">
         <v>1</v>
       </c>
-      <c r="N24" t="s">
+      <c r="O24" t="s">
         <v>42</v>
       </c>
-      <c r="O24" t="s">
+      <c r="R24" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -2635,11 +2710,11 @@
       <c r="J25">
         <v>1</v>
       </c>
-      <c r="O25" t="s">
+      <c r="R25" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>43</v>
       </c>
@@ -2679,11 +2754,20 @@
       <c r="M26" t="s">
         <v>47</v>
       </c>
-      <c r="O26" t="s">
+      <c r="N26" t="s">
+        <v>47</v>
+      </c>
+      <c r="P26" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>47</v>
+      </c>
+      <c r="R26" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -2714,11 +2798,11 @@
       <c r="J27">
         <v>2</v>
       </c>
-      <c r="O27" t="s">
+      <c r="R27" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -2749,14 +2833,14 @@
       <c r="J28">
         <v>2</v>
       </c>
-      <c r="N28" t="s">
+      <c r="O28" t="s">
         <v>48</v>
       </c>
-      <c r="O28" t="s">
+      <c r="R28" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -2787,11 +2871,11 @@
       <c r="J29">
         <v>2</v>
       </c>
-      <c r="O29" t="s">
+      <c r="R29" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -2822,11 +2906,11 @@
       <c r="J30">
         <v>1</v>
       </c>
-      <c r="O30" t="s">
+      <c r="R30" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>50</v>
       </c>
@@ -2857,11 +2941,11 @@
       <c r="J31">
         <v>2</v>
       </c>
-      <c r="O31" t="s">
+      <c r="R31" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -2892,11 +2976,11 @@
       <c r="J32">
         <v>2</v>
       </c>
-      <c r="O32" t="s">
+      <c r="R32" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -2936,11 +3020,20 @@
       <c r="M33" t="s">
         <v>36</v>
       </c>
-      <c r="O33" t="s">
+      <c r="N33" t="s">
+        <v>36</v>
+      </c>
+      <c r="P33" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>36</v>
+      </c>
+      <c r="R33" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>47</v>
       </c>
@@ -2971,11 +3064,11 @@
       <c r="J34">
         <v>2</v>
       </c>
-      <c r="O34" t="s">
+      <c r="R34" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>53</v>
       </c>
@@ -3006,11 +3099,11 @@
       <c r="J35">
         <v>2</v>
       </c>
-      <c r="O35" t="s">
+      <c r="R35" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>54</v>
       </c>
@@ -3041,11 +3134,11 @@
       <c r="J36">
         <v>3</v>
       </c>
-      <c r="O36" t="s">
+      <c r="R36" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -3076,11 +3169,11 @@
       <c r="J37">
         <v>2</v>
       </c>
-      <c r="O37" t="s">
+      <c r="R37" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>55</v>
       </c>
@@ -3111,14 +3204,14 @@
       <c r="J38">
         <v>2</v>
       </c>
-      <c r="N38" t="s">
+      <c r="O38" t="s">
         <v>56</v>
       </c>
-      <c r="O38" t="s">
+      <c r="R38" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>51</v>
       </c>
@@ -3149,11 +3242,11 @@
       <c r="J39">
         <v>3</v>
       </c>
-      <c r="O39" t="s">
+      <c r="R39" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>32</v>
       </c>
@@ -3184,11 +3277,11 @@
       <c r="J40">
         <v>2</v>
       </c>
-      <c r="O40" t="s">
+      <c r="R40" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>36</v>
       </c>
@@ -3219,11 +3312,11 @@
       <c r="J41">
         <v>1</v>
       </c>
-      <c r="O41" t="s">
+      <c r="R41" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>57</v>
       </c>
@@ -3254,14 +3347,14 @@
       <c r="J42">
         <v>2</v>
       </c>
-      <c r="N42" t="s">
+      <c r="O42" t="s">
         <v>41</v>
       </c>
-      <c r="O42" t="s">
+      <c r="R42" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>56</v>
       </c>
@@ -3292,11 +3385,11 @@
       <c r="J43">
         <v>3</v>
       </c>
-      <c r="O43" t="s">
+      <c r="R43" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>58</v>
       </c>
@@ -3336,11 +3429,20 @@
       <c r="M44" t="s">
         <v>46</v>
       </c>
-      <c r="O44" t="s">
+      <c r="N44" t="s">
+        <v>46</v>
+      </c>
+      <c r="P44" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>46</v>
+      </c>
+      <c r="R44" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>61</v>
       </c>
@@ -3381,13 +3483,22 @@
         <v>64</v>
       </c>
       <c r="N45" t="s">
+        <v>64</v>
+      </c>
+      <c r="O45" t="s">
         <v>59</v>
       </c>
-      <c r="O45" t="s">
+      <c r="P45" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>64</v>
+      </c>
+      <c r="R45" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>65</v>
       </c>
@@ -3418,11 +3529,11 @@
       <c r="J46">
         <v>1</v>
       </c>
-      <c r="O46" t="s">
+      <c r="R46" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>41</v>
       </c>
@@ -3453,11 +3564,11 @@
       <c r="J47">
         <v>2</v>
       </c>
-      <c r="O47" t="s">
+      <c r="R47" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>66</v>
       </c>
@@ -3488,11 +3599,11 @@
       <c r="J48">
         <v>2</v>
       </c>
-      <c r="O48" t="s">
+      <c r="R48" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>67</v>
       </c>
@@ -3523,14 +3634,14 @@
       <c r="J49">
         <v>2</v>
       </c>
-      <c r="N49" t="s">
+      <c r="O49" t="s">
         <v>68</v>
       </c>
-      <c r="O49" t="s">
+      <c r="R49" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>59</v>
       </c>
@@ -3561,11 +3672,11 @@
       <c r="J50">
         <v>3</v>
       </c>
-      <c r="O50" t="s">
+      <c r="R50" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>62</v>
       </c>
@@ -3596,11 +3707,11 @@
       <c r="J51">
         <v>2</v>
       </c>
-      <c r="O51" t="s">
+      <c r="R51" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>46</v>
       </c>
@@ -3631,11 +3742,11 @@
       <c r="J52">
         <v>2</v>
       </c>
-      <c r="O52" t="s">
+      <c r="R52" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>64</v>
       </c>
@@ -3666,11 +3777,11 @@
       <c r="J53">
         <v>1</v>
       </c>
-      <c r="O53" t="s">
+      <c r="R53" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>68</v>
       </c>
@@ -3701,11 +3812,11 @@
       <c r="J54">
         <v>1</v>
       </c>
-      <c r="O54" t="s">
+      <c r="R54" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>69</v>
       </c>
@@ -3736,11 +3847,11 @@
       <c r="J55">
         <v>1</v>
       </c>
-      <c r="O55" t="s">
+      <c r="R55" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>70</v>
       </c>
@@ -3771,11 +3882,11 @@
       <c r="J56">
         <v>1</v>
       </c>
-      <c r="O56" t="s">
+      <c r="R56" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>71</v>
       </c>
@@ -3815,11 +3926,20 @@
       <c r="M57" t="s">
         <v>74</v>
       </c>
-      <c r="O57" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N57" t="s">
+        <v>74</v>
+      </c>
+      <c r="P57" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>74</v>
+      </c>
+      <c r="R57" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>75</v>
       </c>
@@ -3850,11 +3970,11 @@
       <c r="J58">
         <v>2</v>
       </c>
-      <c r="O58" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R58" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>52</v>
       </c>
@@ -3885,14 +4005,14 @@
       <c r="J59">
         <v>2</v>
       </c>
-      <c r="N59" t="s">
+      <c r="O59" t="s">
         <v>76</v>
       </c>
-      <c r="O59" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R59" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>77</v>
       </c>
@@ -3932,11 +4052,20 @@
       <c r="M60" t="s">
         <v>80</v>
       </c>
-      <c r="O60" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N60" t="s">
+        <v>80</v>
+      </c>
+      <c r="P60" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>80</v>
+      </c>
+      <c r="R60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>81</v>
       </c>
@@ -3967,11 +4096,11 @@
       <c r="J61">
         <v>1</v>
       </c>
-      <c r="O61" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R61" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>82</v>
       </c>
@@ -4002,11 +4131,11 @@
       <c r="J62">
         <v>2</v>
       </c>
-      <c r="O62" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R62" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>72</v>
       </c>
@@ -4037,14 +4166,14 @@
       <c r="J63">
         <v>2</v>
       </c>
-      <c r="N63" t="s">
+      <c r="O63" t="s">
         <v>80</v>
       </c>
-      <c r="O63" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R63" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>76</v>
       </c>
@@ -4075,11 +4204,11 @@
       <c r="J64">
         <v>1</v>
       </c>
-      <c r="O64" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R64" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>74</v>
       </c>
@@ -4110,11 +4239,11 @@
       <c r="J65">
         <v>2</v>
       </c>
-      <c r="O65" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R65" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>78</v>
       </c>
@@ -4145,11 +4274,11 @@
       <c r="J66">
         <v>1</v>
       </c>
-      <c r="O66" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R66" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>83</v>
       </c>
@@ -4180,11 +4309,11 @@
       <c r="J67">
         <v>2</v>
       </c>
-      <c r="O67" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R67" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>80</v>
       </c>
@@ -4215,11 +4344,11 @@
       <c r="J68">
         <v>2</v>
       </c>
-      <c r="O68" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R68" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>84</v>
       </c>
@@ -4250,14 +4379,14 @@
       <c r="J69">
         <v>2</v>
       </c>
-      <c r="N69" t="s">
+      <c r="O69" t="s">
         <v>85</v>
       </c>
-      <c r="O69" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R69" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>60</v>
       </c>
@@ -4288,11 +4417,11 @@
       <c r="J70">
         <v>1</v>
       </c>
-      <c r="O70" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R70" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>63</v>
       </c>
@@ -4332,11 +4461,20 @@
       <c r="M71" t="s">
         <v>88</v>
       </c>
-      <c r="O71" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N71" t="s">
+        <v>88</v>
+      </c>
+      <c r="P71" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>88</v>
+      </c>
+      <c r="R71" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>89</v>
       </c>
@@ -4367,11 +4505,11 @@
       <c r="J72">
         <v>3</v>
       </c>
-      <c r="O72" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R72" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>90</v>
       </c>
@@ -4402,14 +4540,14 @@
       <c r="J73">
         <v>1</v>
       </c>
-      <c r="N73" t="s">
+      <c r="O73" t="s">
         <v>91</v>
       </c>
-      <c r="O73" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R73" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>85</v>
       </c>
@@ -4440,11 +4578,11 @@
       <c r="J74">
         <v>3</v>
       </c>
-      <c r="O74" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R74" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>92</v>
       </c>
@@ -4475,11 +4613,11 @@
       <c r="J75">
         <v>2</v>
       </c>
-      <c r="O75" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R75" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>93</v>
       </c>
@@ -4510,11 +4648,11 @@
       <c r="J76">
         <v>1</v>
       </c>
-      <c r="O76" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R76" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -4545,11 +4683,11 @@
       <c r="J77">
         <v>2</v>
       </c>
-      <c r="O77" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R77" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>91</v>
       </c>
@@ -4580,11 +4718,11 @@
       <c r="J78">
         <v>1</v>
       </c>
-      <c r="O78" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R78" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>88</v>
       </c>
@@ -4615,11 +4753,11 @@
       <c r="J79">
         <v>1</v>
       </c>
-      <c r="O79" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R79" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>94</v>
       </c>
@@ -4650,11 +4788,11 @@
       <c r="J80">
         <v>2</v>
       </c>
-      <c r="O80" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R80" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>95</v>
       </c>
@@ -4685,11 +4823,11 @@
       <c r="J81">
         <v>1</v>
       </c>
-      <c r="O81" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R81" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>96</v>
       </c>
@@ -4720,11 +4858,11 @@
       <c r="J82">
         <v>2</v>
       </c>
-      <c r="O82" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R82" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>73</v>
       </c>
@@ -4755,14 +4893,14 @@
       <c r="J83">
         <v>1</v>
       </c>
-      <c r="N83" t="s">
+      <c r="O83" t="s">
         <v>97</v>
       </c>
-      <c r="O83" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R83" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>98</v>
       </c>
@@ -4802,11 +4940,20 @@
       <c r="M84" t="s">
         <v>101</v>
       </c>
-      <c r="O84" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N84" t="s">
+        <v>101</v>
+      </c>
+      <c r="P84" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q84" t="s">
+        <v>101</v>
+      </c>
+      <c r="R84" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>102</v>
       </c>
@@ -4837,11 +4984,11 @@
       <c r="J85">
         <v>1</v>
       </c>
-      <c r="O85" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R85" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>79</v>
       </c>
@@ -4872,11 +5019,11 @@
       <c r="J86">
         <v>2</v>
       </c>
-      <c r="O86" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R86" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>103</v>
       </c>
@@ -4907,14 +5054,14 @@
       <c r="J87">
         <v>1</v>
       </c>
-      <c r="N87" t="s">
+      <c r="O87" t="s">
         <v>101</v>
       </c>
-      <c r="O87" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R87" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>97</v>
       </c>
@@ -4945,11 +5092,11 @@
       <c r="J88">
         <v>3</v>
       </c>
-      <c r="O88" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R88" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>104</v>
       </c>
@@ -4980,11 +5127,11 @@
       <c r="J89">
         <v>3</v>
       </c>
-      <c r="O89" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R89" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>99</v>
       </c>
@@ -5015,14 +5162,14 @@
       <c r="J90">
         <v>1</v>
       </c>
-      <c r="N90" t="s">
+      <c r="O90" t="s">
         <v>105</v>
       </c>
-      <c r="O90" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R90" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>106</v>
       </c>
@@ -5053,11 +5200,11 @@
       <c r="J91">
         <v>2</v>
       </c>
-      <c r="O91" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R91" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>101</v>
       </c>
@@ -5088,11 +5235,11 @@
       <c r="J92">
         <v>2</v>
       </c>
-      <c r="O92" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R92" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>107</v>
       </c>
@@ -5123,11 +5270,11 @@
       <c r="J93">
         <v>1</v>
       </c>
-      <c r="O93" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R93" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>108</v>
       </c>
@@ -5158,14 +5305,14 @@
       <c r="J94">
         <v>2</v>
       </c>
-      <c r="N94" t="s">
+      <c r="O94" t="s">
         <v>109</v>
       </c>
-      <c r="O94" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R94" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>105</v>
       </c>
@@ -5196,11 +5343,11 @@
       <c r="J95">
         <v>1</v>
       </c>
-      <c r="O95" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R95" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>110</v>
       </c>
@@ -5231,11 +5378,11 @@
       <c r="J96">
         <v>3</v>
       </c>
-      <c r="O96" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R96" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="97" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>87</v>
       </c>
@@ -5266,11 +5413,11 @@
       <c r="J97">
         <v>2</v>
       </c>
-      <c r="O97" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R97" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="98" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>111</v>
       </c>
@@ -5310,11 +5457,20 @@
       <c r="M98" t="s">
         <v>114</v>
       </c>
-      <c r="O98" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N98" t="s">
+        <v>114</v>
+      </c>
+      <c r="P98" t="s">
+        <v>114</v>
+      </c>
+      <c r="Q98" t="s">
+        <v>114</v>
+      </c>
+      <c r="R98" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="99" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>109</v>
       </c>
@@ -5345,11 +5501,11 @@
       <c r="J99">
         <v>2</v>
       </c>
-      <c r="O99" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R99" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="100" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>115</v>
       </c>
@@ -5380,11 +5536,11 @@
       <c r="J100">
         <v>2</v>
       </c>
-      <c r="O100" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R100" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="101" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>116</v>
       </c>
@@ -5424,11 +5580,20 @@
       <c r="M101" t="s">
         <v>119</v>
       </c>
-      <c r="O101" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N101" t="s">
+        <v>119</v>
+      </c>
+      <c r="P101" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q101" t="s">
+        <v>119</v>
+      </c>
+      <c r="R101" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="102" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>120</v>
       </c>
@@ -5459,11 +5624,11 @@
       <c r="J102">
         <v>2</v>
       </c>
-      <c r="O102" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R102" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="103" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>121</v>
       </c>
@@ -5494,11 +5659,11 @@
       <c r="J103">
         <v>2</v>
       </c>
-      <c r="O103" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R103" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="104" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>112</v>
       </c>
@@ -5529,14 +5694,14 @@
       <c r="J104">
         <v>1</v>
       </c>
-      <c r="N104" t="s">
+      <c r="O104" t="s">
         <v>119</v>
       </c>
-      <c r="O104" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R104" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="105" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>122</v>
       </c>
@@ -5567,11 +5732,11 @@
       <c r="J105">
         <v>1</v>
       </c>
-      <c r="O105" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R105" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="106" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>114</v>
       </c>
@@ -5602,11 +5767,11 @@
       <c r="J106">
         <v>1</v>
       </c>
-      <c r="O106" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R106" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="107" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>117</v>
       </c>
@@ -5637,11 +5802,11 @@
       <c r="J107">
         <v>1</v>
       </c>
-      <c r="O107" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R107" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="108" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>123</v>
       </c>
@@ -5672,14 +5837,14 @@
       <c r="J108">
         <v>2</v>
       </c>
-      <c r="N108" t="s">
+      <c r="O108" t="s">
         <v>124</v>
       </c>
-      <c r="O108" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R108" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="109" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>119</v>
       </c>
@@ -5710,11 +5875,11 @@
       <c r="J109">
         <v>1</v>
       </c>
-      <c r="O109" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R109" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="110" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>100</v>
       </c>
@@ -5745,11 +5910,11 @@
       <c r="J110">
         <v>1</v>
       </c>
-      <c r="O110" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R110" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="111" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>125</v>
       </c>
@@ -5789,11 +5954,20 @@
       <c r="M111" t="s">
         <v>128</v>
       </c>
-      <c r="O111" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N111" t="s">
+        <v>128</v>
+      </c>
+      <c r="P111" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q111" t="s">
+        <v>128</v>
+      </c>
+      <c r="R111" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="112" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>129</v>
       </c>
@@ -5824,11 +5998,11 @@
       <c r="J112">
         <v>2</v>
       </c>
-      <c r="O112" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R112" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="113" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>124</v>
       </c>
@@ -5859,11 +6033,11 @@
       <c r="J113">
         <v>1</v>
       </c>
-      <c r="O113" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R113" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="114" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>130</v>
       </c>
@@ -5894,11 +6068,11 @@
       <c r="J114">
         <v>2</v>
       </c>
-      <c r="O114" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R114" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="115" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>131</v>
       </c>
@@ -5929,14 +6103,14 @@
       <c r="J115">
         <v>2</v>
       </c>
-      <c r="N115" t="s">
+      <c r="O115" t="s">
         <v>132</v>
       </c>
-      <c r="O115" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R115" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="116" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>133</v>
       </c>
@@ -5967,11 +6141,11 @@
       <c r="J116">
         <v>2</v>
       </c>
-      <c r="O116" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R116" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="117" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>126</v>
       </c>
@@ -6002,11 +6176,11 @@
       <c r="J117">
         <v>1</v>
       </c>
-      <c r="O117" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R117" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="118" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>134</v>
       </c>
@@ -6037,11 +6211,11 @@
       <c r="J118">
         <v>2</v>
       </c>
-      <c r="O118" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R118" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="119" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>128</v>
       </c>
@@ -6072,14 +6246,14 @@
       <c r="J119">
         <v>1</v>
       </c>
-      <c r="N119" t="s">
+      <c r="O119" t="s">
         <v>113</v>
       </c>
-      <c r="O119" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R119" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="120" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>132</v>
       </c>
@@ -6110,11 +6284,11 @@
       <c r="J120">
         <v>3</v>
       </c>
-      <c r="O120" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R120" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="121" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>135</v>
       </c>
@@ -6145,11 +6319,11 @@
       <c r="J121">
         <v>1</v>
       </c>
-      <c r="O121" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R121" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="122" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>136</v>
       </c>
@@ -6189,11 +6363,20 @@
       <c r="M122" t="s">
         <v>139</v>
       </c>
-      <c r="O122" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N122" t="s">
+        <v>139</v>
+      </c>
+      <c r="P122" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q122" t="s">
+        <v>139</v>
+      </c>
+      <c r="R122" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="123" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>140</v>
       </c>
@@ -6233,11 +6416,20 @@
       <c r="M123" t="s">
         <v>143</v>
       </c>
-      <c r="O123" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N123" t="s">
+        <v>143</v>
+      </c>
+      <c r="P123" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q123" t="s">
+        <v>143</v>
+      </c>
+      <c r="R123" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="124" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>113</v>
       </c>
@@ -6268,11 +6460,11 @@
       <c r="J124">
         <v>2</v>
       </c>
-      <c r="O124" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R124" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="125" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>144</v>
       </c>
@@ -6303,11 +6495,11 @@
       <c r="J125">
         <v>1</v>
       </c>
-      <c r="O125" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R125" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="126" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>145</v>
       </c>
@@ -6338,11 +6530,11 @@
       <c r="J126">
         <v>1</v>
       </c>
-      <c r="O126" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R126" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="127" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>118</v>
       </c>
@@ -6373,11 +6565,11 @@
       <c r="J127">
         <v>2</v>
       </c>
-      <c r="O127" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R127" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="128" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>137</v>
       </c>
@@ -6408,11 +6600,11 @@
       <c r="J128">
         <v>1</v>
       </c>
-      <c r="O128" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R128" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="129" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>141</v>
       </c>
@@ -6443,14 +6635,14 @@
       <c r="J129">
         <v>2</v>
       </c>
-      <c r="N129" t="s">
+      <c r="O129" t="s">
         <v>146</v>
       </c>
-      <c r="O129" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R129" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="130" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>139</v>
       </c>
@@ -6481,11 +6673,11 @@
       <c r="J130">
         <v>2</v>
       </c>
-      <c r="O130" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R130" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="131" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>143</v>
       </c>
@@ -6516,11 +6708,11 @@
       <c r="J131">
         <v>2</v>
       </c>
-      <c r="O131" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R131" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="132" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>147</v>
       </c>
@@ -6551,11 +6743,11 @@
       <c r="J132">
         <v>2</v>
       </c>
-      <c r="O132" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R132" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="133" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>148</v>
       </c>
@@ -6586,14 +6778,14 @@
       <c r="J133">
         <v>2</v>
       </c>
-      <c r="N133" t="s">
+      <c r="O133" t="s">
         <v>149</v>
       </c>
-      <c r="O133" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R133" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="134" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>146</v>
       </c>
@@ -6624,11 +6816,11 @@
       <c r="J134">
         <v>1</v>
       </c>
-      <c r="O134" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R134" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="135" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>150</v>
       </c>
@@ -6668,11 +6860,20 @@
       <c r="M135" t="s">
         <v>153</v>
       </c>
-      <c r="O135" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N135" t="s">
+        <v>153</v>
+      </c>
+      <c r="P135" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q135" t="s">
+        <v>153</v>
+      </c>
+      <c r="R135" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="136" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>154</v>
       </c>
@@ -6703,11 +6904,11 @@
       <c r="J136">
         <v>2</v>
       </c>
-      <c r="O136" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R136" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="137" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>127</v>
       </c>
@@ -6738,11 +6939,11 @@
       <c r="J137">
         <v>2</v>
       </c>
-      <c r="O137" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R137" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="138" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>149</v>
       </c>
@@ -6773,11 +6974,11 @@
       <c r="J138">
         <v>1</v>
       </c>
-      <c r="O138" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R138" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="139" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>155</v>
       </c>
@@ -6808,14 +7009,14 @@
       <c r="J139">
         <v>2</v>
       </c>
-      <c r="N139" t="s">
+      <c r="O139" t="s">
         <v>156</v>
       </c>
-      <c r="O139" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R139" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="140" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>157</v>
       </c>
@@ -6837,8 +7038,8 @@
       <c r="G140">
         <v>0</v>
       </c>
-      <c r="H140" t="s">
-        <v>260</v>
+      <c r="H140">
+        <v>1</v>
       </c>
       <c r="I140">
         <v>1</v>
@@ -6846,14 +7047,14 @@
       <c r="J140">
         <v>1</v>
       </c>
-      <c r="N140" t="s">
+      <c r="O140" t="s">
         <v>158</v>
       </c>
-      <c r="O140" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R140" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="141" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>151</v>
       </c>
@@ -6884,11 +7085,11 @@
       <c r="J141">
         <v>2</v>
       </c>
-      <c r="O141" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R141" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="142" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>159</v>
       </c>
@@ -6919,11 +7120,11 @@
       <c r="J142">
         <v>1</v>
       </c>
-      <c r="O142" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R142" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="143" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>153</v>
       </c>
@@ -6954,11 +7155,11 @@
       <c r="J143">
         <v>1</v>
       </c>
-      <c r="O143" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R143" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="144" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>156</v>
       </c>
@@ -6989,14 +7190,14 @@
       <c r="J144">
         <v>2</v>
       </c>
-      <c r="N144" t="s">
+      <c r="O144" t="s">
         <v>142</v>
       </c>
-      <c r="O144" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R144" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="145" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>158</v>
       </c>
@@ -7027,11 +7228,11 @@
       <c r="J145">
         <v>3</v>
       </c>
-      <c r="O145" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R145" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="146" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>160</v>
       </c>
@@ -7062,11 +7263,11 @@
       <c r="J146">
         <v>2</v>
       </c>
-      <c r="O146" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R146" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="147" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>161</v>
       </c>
@@ -7097,11 +7298,11 @@
       <c r="J147">
         <v>2</v>
       </c>
-      <c r="O147" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R147" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="148" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>138</v>
       </c>
@@ -7141,11 +7342,20 @@
       <c r="M148" t="s">
         <v>164</v>
       </c>
-      <c r="O148" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N148" t="s">
+        <v>164</v>
+      </c>
+      <c r="P148" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q148" t="s">
+        <v>164</v>
+      </c>
+      <c r="R148" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="149" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>142</v>
       </c>
@@ -7176,11 +7386,11 @@
       <c r="J149">
         <v>1</v>
       </c>
-      <c r="O149" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R149" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="150" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>165</v>
       </c>
@@ -7211,11 +7421,11 @@
       <c r="J150">
         <v>2</v>
       </c>
-      <c r="O150" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R150" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="151" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>166</v>
       </c>
@@ -7246,11 +7456,11 @@
       <c r="J151">
         <v>1</v>
       </c>
-      <c r="O151" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R151" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="152" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>167</v>
       </c>
@@ -7281,11 +7491,11 @@
       <c r="J152">
         <v>1</v>
       </c>
-      <c r="O152" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R152" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="153" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>168</v>
       </c>
@@ -7316,11 +7526,11 @@
       <c r="J153">
         <v>2</v>
       </c>
-      <c r="O153" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R153" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="154" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>162</v>
       </c>
@@ -7351,14 +7561,14 @@
       <c r="J154">
         <v>1</v>
       </c>
-      <c r="N154" t="s">
+      <c r="O154" t="s">
         <v>169</v>
       </c>
-      <c r="O154" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R154" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="155" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>170</v>
       </c>
@@ -7389,11 +7599,11 @@
       <c r="J155">
         <v>2</v>
       </c>
-      <c r="O155" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R155" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="156" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>164</v>
       </c>
@@ -7424,11 +7634,11 @@
       <c r="J156">
         <v>2</v>
       </c>
-      <c r="O156" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R156" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="157" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>171</v>
       </c>
@@ -7459,11 +7669,11 @@
       <c r="J157">
         <v>2</v>
       </c>
-      <c r="O157" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R157" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="158" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>172</v>
       </c>
@@ -7494,14 +7704,14 @@
       <c r="J158">
         <v>2</v>
       </c>
-      <c r="N158" t="s">
+      <c r="O158" t="s">
         <v>173</v>
       </c>
-      <c r="O158" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R158" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="159" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>169</v>
       </c>
@@ -7541,11 +7751,20 @@
       <c r="M159" t="s">
         <v>176</v>
       </c>
-      <c r="O159" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N159" t="s">
+        <v>176</v>
+      </c>
+      <c r="P159" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q159" t="s">
+        <v>176</v>
+      </c>
+      <c r="R159" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="160" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>177</v>
       </c>
@@ -7585,11 +7804,20 @@
       <c r="M160" t="s">
         <v>180</v>
       </c>
-      <c r="O160" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N160" t="s">
+        <v>180</v>
+      </c>
+      <c r="P160" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q160" t="s">
+        <v>180</v>
+      </c>
+      <c r="R160" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="161" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>152</v>
       </c>
@@ -7620,11 +7848,11 @@
       <c r="J161">
         <v>2</v>
       </c>
-      <c r="O161" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R161" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="162" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>181</v>
       </c>
@@ -7655,11 +7883,11 @@
       <c r="J162">
         <v>1</v>
       </c>
-      <c r="O162" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R162" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="163" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>173</v>
       </c>
@@ -7690,11 +7918,11 @@
       <c r="J163">
         <v>1</v>
       </c>
-      <c r="O163" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R163" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="164" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>182</v>
       </c>
@@ -7725,11 +7953,11 @@
       <c r="J164">
         <v>2</v>
       </c>
-      <c r="O164" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R164" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="165" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>174</v>
       </c>
@@ -7760,11 +7988,11 @@
       <c r="J165">
         <v>2</v>
       </c>
-      <c r="O165" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R165" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="166" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>178</v>
       </c>
@@ -7795,11 +8023,11 @@
       <c r="J166">
         <v>2</v>
       </c>
-      <c r="O166" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R166" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="167" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>176</v>
       </c>
@@ -7830,11 +8058,11 @@
       <c r="J167">
         <v>2</v>
       </c>
-      <c r="O167" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R167" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="168" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>180</v>
       </c>
@@ -7865,11 +8093,11 @@
       <c r="J168">
         <v>2</v>
       </c>
-      <c r="O168" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R168" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="169" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>183</v>
       </c>
@@ -7900,11 +8128,11 @@
       <c r="J169">
         <v>2</v>
       </c>
-      <c r="O169" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R169" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="170" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>184</v>
       </c>
@@ -7935,14 +8163,14 @@
       <c r="J170">
         <v>1</v>
       </c>
-      <c r="N170" t="s">
+      <c r="O170" t="s">
         <v>185</v>
       </c>
-      <c r="O170" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R170" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="171" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>186</v>
       </c>
@@ -7973,11 +8201,11 @@
       <c r="J171">
         <v>2</v>
       </c>
-      <c r="O171" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R171" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="172" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>187</v>
       </c>
@@ -8017,11 +8245,20 @@
       <c r="M172" t="s">
         <v>190</v>
       </c>
-      <c r="O172" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N172" t="s">
+        <v>190</v>
+      </c>
+      <c r="P172" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q172" t="s">
+        <v>190</v>
+      </c>
+      <c r="R172" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="173" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>191</v>
       </c>
@@ -8052,11 +8289,11 @@
       <c r="J173">
         <v>1</v>
       </c>
-      <c r="O173" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R173" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="174" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>163</v>
       </c>
@@ -8087,14 +8324,14 @@
       <c r="J174">
         <v>2</v>
       </c>
-      <c r="N174" t="s">
+      <c r="O174" t="s">
         <v>192</v>
       </c>
-      <c r="O174" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R174" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="175" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>185</v>
       </c>
@@ -8125,11 +8362,11 @@
       <c r="J175">
         <v>1</v>
       </c>
-      <c r="O175" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R175" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="176" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>193</v>
       </c>
@@ -8160,11 +8397,11 @@
       <c r="J176">
         <v>2</v>
       </c>
-      <c r="O176" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R176" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="177" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>194</v>
       </c>
@@ -8195,11 +8432,11 @@
       <c r="J177">
         <v>1</v>
       </c>
-      <c r="O177" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R177" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="178" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>188</v>
       </c>
@@ -8230,11 +8467,11 @@
       <c r="J178">
         <v>1</v>
       </c>
-      <c r="O178" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R178" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="179" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>192</v>
       </c>
@@ -8265,11 +8502,11 @@
       <c r="J179">
         <v>2</v>
       </c>
-      <c r="O179" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R179" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="180" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>190</v>
       </c>
@@ -8300,11 +8537,11 @@
       <c r="J180">
         <v>1</v>
       </c>
-      <c r="O180" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R180" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="181" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>195</v>
       </c>
@@ -8335,11 +8572,11 @@
       <c r="J181">
         <v>1</v>
       </c>
-      <c r="O181" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R181" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="182" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>196</v>
       </c>
@@ -8370,11 +8607,11 @@
       <c r="J182">
         <v>3</v>
       </c>
-      <c r="O182" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R182" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="183" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>197</v>
       </c>
@@ -8405,11 +8642,11 @@
       <c r="J183">
         <v>2</v>
       </c>
-      <c r="O183" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R183" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="184" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>198</v>
       </c>
@@ -8440,14 +8677,14 @@
       <c r="J184">
         <v>1</v>
       </c>
-      <c r="N184" t="s">
+      <c r="O184" t="s">
         <v>199</v>
       </c>
-      <c r="O184" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R184" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="185" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>175</v>
       </c>
@@ -8478,11 +8715,11 @@
       <c r="J185">
         <v>1</v>
       </c>
-      <c r="O185" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R185" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="186" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>179</v>
       </c>
@@ -8513,11 +8750,11 @@
       <c r="J186">
         <v>3</v>
       </c>
-      <c r="O186" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R186" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="187" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>200</v>
       </c>
@@ -8548,11 +8785,11 @@
       <c r="J187">
         <v>2</v>
       </c>
-      <c r="O187" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R187" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="188" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>201</v>
       </c>
@@ -8583,14 +8820,14 @@
       <c r="J188">
         <v>1</v>
       </c>
-      <c r="N188" t="s">
+      <c r="O188" t="s">
         <v>202</v>
       </c>
-      <c r="O188" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R188" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="189" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>199</v>
       </c>
@@ -8621,11 +8858,11 @@
       <c r="J189">
         <v>2</v>
       </c>
-      <c r="O189" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R189" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="190" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>203</v>
       </c>
@@ -8656,11 +8893,11 @@
       <c r="J190">
         <v>1</v>
       </c>
-      <c r="O190" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R190" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="191" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>204</v>
       </c>
@@ -8691,11 +8928,11 @@
       <c r="J191">
         <v>1</v>
       </c>
-      <c r="O191" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R191" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="192" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>205</v>
       </c>
@@ -8735,11 +8972,20 @@
       <c r="M192" t="s">
         <v>207</v>
       </c>
-      <c r="O192" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N192" t="s">
+        <v>207</v>
+      </c>
+      <c r="P192" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q192" t="s">
+        <v>207</v>
+      </c>
+      <c r="R192" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="193" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>202</v>
       </c>
@@ -8770,11 +9016,11 @@
       <c r="J193">
         <v>1</v>
       </c>
-      <c r="O193" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R193" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="194" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>208</v>
       </c>
@@ -8805,11 +9051,11 @@
       <c r="J194">
         <v>1</v>
       </c>
-      <c r="O194" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R194" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="195" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>209</v>
       </c>
@@ -8840,11 +9086,11 @@
       <c r="J195">
         <v>2</v>
       </c>
-      <c r="O195" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R195" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="196" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>210</v>
       </c>
@@ -8875,11 +9121,11 @@
       <c r="J196">
         <v>2</v>
       </c>
-      <c r="O196" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R196" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="197" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>211</v>
       </c>
@@ -8910,11 +9156,11 @@
       <c r="J197">
         <v>3</v>
       </c>
-      <c r="O197" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R197" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="198" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>189</v>
       </c>
@@ -8945,11 +9191,11 @@
       <c r="J198">
         <v>2</v>
       </c>
-      <c r="O198" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R198" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="199" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>212</v>
       </c>
@@ -8980,11 +9226,11 @@
       <c r="J199">
         <v>1</v>
       </c>
-      <c r="O199" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R199" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="200" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>207</v>
       </c>
@@ -9024,11 +9270,20 @@
       <c r="M200" t="s">
         <v>215</v>
       </c>
-      <c r="O200" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N200" t="s">
+        <v>215</v>
+      </c>
+      <c r="P200" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q200" t="s">
+        <v>215</v>
+      </c>
+      <c r="R200" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="201" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>216</v>
       </c>
@@ -9059,11 +9314,11 @@
       <c r="J201">
         <v>2</v>
       </c>
-      <c r="O201" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R201" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="202" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>217</v>
       </c>
@@ -9094,11 +9349,11 @@
       <c r="J202">
         <v>1</v>
       </c>
-      <c r="O202" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R202" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="203" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>218</v>
       </c>
@@ -9129,11 +9384,11 @@
       <c r="J203">
         <v>3</v>
       </c>
-      <c r="O203" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R203" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="204" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>219</v>
       </c>
@@ -9164,11 +9419,11 @@
       <c r="J204">
         <v>1</v>
       </c>
-      <c r="O204" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R204" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="205" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>220</v>
       </c>
@@ -9199,11 +9454,11 @@
       <c r="J205">
         <v>2</v>
       </c>
-      <c r="O205" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R205" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="206" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>213</v>
       </c>
@@ -9234,11 +9489,11 @@
       <c r="J206">
         <v>3</v>
       </c>
-      <c r="O206" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R206" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="207" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>221</v>
       </c>
@@ -9269,11 +9524,11 @@
       <c r="J207">
         <v>2</v>
       </c>
-      <c r="O207" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R207" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="208" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>215</v>
       </c>
@@ -9304,11 +9559,11 @@
       <c r="J208">
         <v>1</v>
       </c>
-      <c r="O208" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R208" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="209" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>222</v>
       </c>
@@ -9339,11 +9594,11 @@
       <c r="J209">
         <v>1</v>
       </c>
-      <c r="O209" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R209" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="210" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>223</v>
       </c>
@@ -9374,11 +9629,11 @@
       <c r="J210">
         <v>2</v>
       </c>
-      <c r="O210" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R210" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="211" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>224</v>
       </c>
@@ -9416,13 +9671,22 @@
         <v>226</v>
       </c>
       <c r="N211" t="s">
+        <v>226</v>
+      </c>
+      <c r="O211" t="s">
         <v>227</v>
       </c>
-      <c r="O211" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P211" t="s">
+        <v>226</v>
+      </c>
+      <c r="Q211" t="s">
+        <v>226</v>
+      </c>
+      <c r="R211" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="212" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>228</v>
       </c>
@@ -9459,11 +9723,20 @@
       <c r="M212" t="s">
         <v>229</v>
       </c>
-      <c r="O212" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N212" t="s">
+        <v>229</v>
+      </c>
+      <c r="P212" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q212" t="s">
+        <v>229</v>
+      </c>
+      <c r="R212" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="213" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>230</v>
       </c>
@@ -9494,11 +9767,11 @@
       <c r="J213">
         <v>2</v>
       </c>
-      <c r="O213" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R213" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="214" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>231</v>
       </c>
@@ -9529,11 +9802,11 @@
       <c r="J214">
         <v>2</v>
       </c>
-      <c r="O214" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R214" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="215" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>232</v>
       </c>
@@ -9564,14 +9837,14 @@
       <c r="J215">
         <v>3</v>
       </c>
-      <c r="N215" t="s">
+      <c r="O215" t="s">
         <v>229</v>
       </c>
-      <c r="O215" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R215" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="216" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>227</v>
       </c>
@@ -9602,11 +9875,11 @@
       <c r="J216">
         <v>2</v>
       </c>
-      <c r="O216" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R216" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="217" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>225</v>
       </c>
@@ -9637,11 +9910,11 @@
       <c r="J217">
         <v>3</v>
       </c>
-      <c r="O217" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R217" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="218" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>206</v>
       </c>
@@ -9672,11 +9945,11 @@
       <c r="J218">
         <v>1</v>
       </c>
-      <c r="O218" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R218" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="219" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>226</v>
       </c>
@@ -9707,11 +9980,11 @@
       <c r="J219">
         <v>2</v>
       </c>
-      <c r="O219" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R219" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="220" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>229</v>
       </c>
@@ -9742,11 +10015,11 @@
       <c r="J220">
         <v>1</v>
       </c>
-      <c r="O220" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R220" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="221" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>233</v>
       </c>
@@ -9777,11 +10050,11 @@
       <c r="J221">
         <v>2</v>
       </c>
-      <c r="O221" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R221" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="222" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>234</v>
       </c>
@@ -9812,11 +10085,11 @@
       <c r="J222">
         <v>1</v>
       </c>
-      <c r="O222" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R222" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="223" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>235</v>
       </c>
@@ -9847,11 +10120,11 @@
       <c r="J223">
         <v>1</v>
       </c>
-      <c r="O223" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R223" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="224" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>236</v>
       </c>
@@ -9888,11 +10161,20 @@
       <c r="M224" t="s">
         <v>238</v>
       </c>
-      <c r="O224" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="225" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="N224" t="s">
+        <v>238</v>
+      </c>
+      <c r="P224" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q224" t="s">
+        <v>238</v>
+      </c>
+      <c r="R224" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="225" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>239</v>
       </c>
@@ -9923,14 +10205,14 @@
       <c r="J225">
         <v>2</v>
       </c>
-      <c r="N225" t="s">
+      <c r="O225" t="s">
         <v>237</v>
       </c>
-      <c r="O225" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="226" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R225" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="226" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>214</v>
       </c>
@@ -9961,11 +10243,11 @@
       <c r="J226">
         <v>1</v>
       </c>
-      <c r="O226" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="227" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R226" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="227" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>240</v>
       </c>
@@ -9996,11 +10278,11 @@
       <c r="J227">
         <v>1</v>
       </c>
-      <c r="O227" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="228" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R227" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="228" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>241</v>
       </c>
@@ -10031,11 +10313,11 @@
       <c r="J228">
         <v>1</v>
       </c>
-      <c r="O228" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="229" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R228" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="229" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>242</v>
       </c>
@@ -10066,14 +10348,14 @@
       <c r="J229">
         <v>2</v>
       </c>
-      <c r="N229" t="s">
+      <c r="O229" t="s">
         <v>243</v>
       </c>
-      <c r="O229" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="230" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R229" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="230" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>237</v>
       </c>
@@ -10104,11 +10386,11 @@
       <c r="J230">
         <v>1</v>
       </c>
-      <c r="O230" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="231" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R230" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="231" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>244</v>
       </c>
@@ -10139,11 +10421,11 @@
       <c r="J231">
         <v>1</v>
       </c>
-      <c r="O231" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="232" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R231" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="232" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>238</v>
       </c>
@@ -10174,11 +10456,11 @@
       <c r="J232">
         <v>1</v>
       </c>
-      <c r="O232" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="233" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R232" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="233" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>245</v>
       </c>
@@ -10209,11 +10491,11 @@
       <c r="J233">
         <v>2</v>
       </c>
-      <c r="O233" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="234" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="R233" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="234" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>243</v>
       </c>
@@ -10244,14 +10526,15 @@
       <c r="J234">
         <v>2</v>
       </c>
-      <c r="O234" t="s">
-        <v>249</v>
+      <c r="R234" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N234" xr:uid="{041A12D7-D1F2-5E4A-959D-815F4F1F9005}"/>
+  <autoFilter ref="A1:O234" xr:uid="{041A12D7-D1F2-5E4A-959D-815F4F1F9005}"/>
+  <phoneticPr fontId="18" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:N1048576" xr:uid="{836F0146-E07F-2A4C-BD11-FE221837FD18}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:Q1048576" xr:uid="{836F0146-E07F-2A4C-BD11-FE221837FD18}">
       <formula1>$A:$A</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>